<commit_message>
Add breadcrumb + logo-strip blocks; resolve lazy-loaded images
- breadcrumb: URL-path-driven auto-block on interior content pages
  (Investment > parent > current), wired via buildAutoBlocks in scripts.js
- logo-strip: block for the partner-logo band on responsible-ownership
- images transformer: resolve lazy-loaded core-image (data-cmp-src) to the
  canonical DAM path before block discovery, so the real asset is captured
  instead of a transient blob: URL
- add logo-strip to the DA block library showcase

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="86">
   <si>
     <t>_reportFile</t>
   </si>
@@ -76,142 +76,160 @@
     <t>investment/about-us.report.json</t>
   </si>
   <si>
+    <t>["cards-explore","columns-split","columns-split","cards-feature","cards-feature"]</t>
+  </si>
+  <si>
+    <t>investment/about-us</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:34:54.320Z</t>
+  </si>
+  <si>
+    <t>About us | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/about-us</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach.report.json</t>
+  </si>
+  <si>
+    <t>["columns-split","columns-split","columns-split","cards-feature","accordion-cards","cards-nav"]</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:35:12.838Z</t>
+  </si>
+  <si>
+    <t>Our investment approach | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach</t>
+  </si>
+  <si>
+    <t>investment/privacy-uk.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>investment/privacy-uk</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:37:22.277Z</t>
+  </si>
+  <si>
+    <t>Privacy Notice | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/privacy-uk</t>
+  </si>
+  <si>
+    <t>investment/what-we-invest-in.report.json</t>
+  </si>
+  <si>
+    <t>["columns-split","columns-split","columns-split","cards-nav"]</t>
+  </si>
+  <si>
+    <t>investment/what-we-invest-in</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:36:16.741Z</t>
+  </si>
+  <si>
+    <t>What we invest in | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/what-we-invest-in</t>
+  </si>
+  <si>
+    <t>investment/about-us/contact-us.report.json</t>
+  </si>
+  <si>
     <t>["cards-nav"]</t>
   </si>
   <si>
-    <t>investment/about-us</t>
-  </si>
-  <si>
-    <t>content-page</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:43:02.786Z</t>
-  </si>
-  <si>
-    <t>About us | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/about-us</t>
-  </si>
-  <si>
-    <t>investment/our-investment-approach.report.json</t>
+    <t>investment/about-us/contact-us</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:35:00.097Z</t>
+  </si>
+  <si>
+    <t>Contact us | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/about-us/contact-us</t>
+  </si>
+  <si>
+    <t>investment/about-us/our-people.report.json</t>
+  </si>
+  <si>
+    <t>["cards-explore","cards-nav"]</t>
+  </si>
+  <si>
+    <t>investment/about-us/our-people</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:35:06.693Z</t>
+  </si>
+  <si>
+    <t>Our people | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/about-us/our-people</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach/investment-strategy.report.json</t>
+  </si>
+  <si>
+    <t>["columns-split","cards-nav"]</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach/investment-strategy</t>
+  </si>
+  <si>
+    <t>2026-08-19T07:35:18.521Z</t>
+  </si>
+  <si>
+    <t>Our investment strategy | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach/investment-strategy</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach/responsible-ownership.report.json</t>
+  </si>
+  <si>
+    <t>["logo-strip","cards-explore","columns-split","cards-nav"]</t>
+  </si>
+  <si>
+    <t>investment/our-investment-approach/responsible-ownership</t>
+  </si>
+  <si>
+    <t>2026-08-19T08:06:30.187Z</t>
+  </si>
+  <si>
+    <t>Responsible Ownership | Investments</t>
+  </si>
+  <si>
+    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach/responsible-ownership</t>
+  </si>
+  <si>
+    <t>investment/what-we-invest-in/infrastructure.report.json</t>
   </si>
   <si>
     <t>["cards-feature","accordion-cards","cards-nav"]</t>
   </si>
   <si>
-    <t>investment/our-investment-approach</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:44:07.307Z</t>
-  </si>
-  <si>
-    <t>Our investment approach | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach</t>
-  </si>
-  <si>
-    <t>investment/privacy-uk.report.json</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>investment/privacy-uk</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:47:52.788Z</t>
-  </si>
-  <si>
-    <t>Privacy Notice | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/privacy-uk</t>
-  </si>
-  <si>
-    <t>investment/what-we-invest-in.report.json</t>
-  </si>
-  <si>
-    <t>investment/what-we-invest-in</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:45:58.596Z</t>
-  </si>
-  <si>
-    <t>What we invest in | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/what-we-invest-in</t>
-  </si>
-  <si>
-    <t>investment/about-us/contact-us.report.json</t>
-  </si>
-  <si>
-    <t>investment/about-us/contact-us</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:43:07.833Z</t>
-  </si>
-  <si>
-    <t>Contact us | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/about-us/contact-us</t>
-  </si>
-  <si>
-    <t>investment/about-us/our-people.report.json</t>
-  </si>
-  <si>
-    <t>investment/about-us/our-people</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:44:01.306Z</t>
-  </si>
-  <si>
-    <t>Our people | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/about-us/our-people</t>
-  </si>
-  <si>
-    <t>investment/our-investment-approach/investment-strategy.report.json</t>
-  </si>
-  <si>
-    <t>investment/our-investment-approach/investment-strategy</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:44:59.135Z</t>
-  </si>
-  <si>
-    <t>Our investment strategy | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach/investment-strategy</t>
-  </si>
-  <si>
-    <t>investment/our-investment-approach/responsible-ownership.report.json</t>
-  </si>
-  <si>
-    <t>investment/our-investment-approach/responsible-ownership</t>
-  </si>
-  <si>
-    <t>2026-08-18T12:45:52.856Z</t>
-  </si>
-  <si>
-    <t>Responsible Ownership | Investments</t>
-  </si>
-  <si>
-    <t>https://awareinvestments.aware.com.au/investment/our-investment-approach/responsible-ownership</t>
-  </si>
-  <si>
-    <t>investment/what-we-invest-in/infrastructure.report.json</t>
-  </si>
-  <si>
     <t>investment/what-we-invest-in/infrastructure</t>
   </si>
   <si>
-    <t>2026-08-18T12:42:57.227Z</t>
+    <t>2026-08-19T07:34:48.222Z</t>
   </si>
   <si>
     <t>Infrastructure | Investments</t>
@@ -229,7 +247,7 @@
     <t>investment/what-we-invest-in/private-equity</t>
   </si>
   <si>
-    <t>2026-08-18T12:46:05.133Z</t>
+    <t>2026-08-19T07:36:21.806Z</t>
   </si>
   <si>
     <t>Private equity | Investments</t>
@@ -244,7 +262,7 @@
     <t>investment/what-we-invest-in/property</t>
   </si>
   <si>
-    <t>2026-08-18T12:46:59.270Z</t>
+    <t>2026-08-19T07:37:15.015Z</t>
   </si>
   <si>
     <t>Property | Investments</t>
@@ -810,10 +828,10 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -822,24 +840,24 @@
         <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -848,24 +866,24 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -874,24 +892,24 @@
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -900,24 +918,24 @@
         <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -926,24 +944,24 @@
         <v>23</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G11" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -952,24 +970,24 @@
         <v>23</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -978,24 +996,24 @@
         <v>23</v>
       </c>
       <c r="F13" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H13" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1004,13 +1022,13 @@
         <v>23</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Package title hero as an authorable hero-banner block with image placement
Turn the 50/50 page-title hero into a proper block so authors control it:
- blocks/hero-banner: magenta title card + hero image, with image-left /
  image-right placement options (defaults to image-right)
- import parser + content-page mapping for the leading .banner section;
  re-imported our-investment-approach and what-we-invest-in to use the block
- scripts.js: leave hero-banner pages to the block; keep the plain magenta
  band only for text-only title sections (About us etc.)
- drop the now-superseded .banner-hero CSS; add hero-banner to the block library

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -97,13 +97,13 @@
     <t>investment/our-investment-approach.report.json</t>
   </si>
   <si>
-    <t>["columns-split","columns-split","columns-split","cards-feature","accordion-cards","cards-nav"]</t>
+    <t>["hero-banner","columns-split","columns-split","columns-split","cards-feature","accordion-cards","cards-nav"]</t>
   </si>
   <si>
     <t>investment/our-investment-approach</t>
   </si>
   <si>
-    <t>2026-08-19T07:35:12.838Z</t>
+    <t>2026-08-20T00:52:11.855Z</t>
   </si>
   <si>
     <t>Our investment approach | Investments</t>
@@ -133,13 +133,13 @@
     <t>investment/what-we-invest-in.report.json</t>
   </si>
   <si>
-    <t>["columns-split","columns-split","columns-split","cards-nav"]</t>
+    <t>["hero-banner","columns-split","columns-split","columns-split","cards-nav"]</t>
   </si>
   <si>
     <t>investment/what-we-invest-in</t>
   </si>
   <si>
-    <t>2026-08-19T07:36:16.741Z</t>
+    <t>2026-08-20T00:53:04.974Z</t>
   </si>
   <si>
     <t>What we invest in | Investments</t>

</xml_diff>